<commit_message>
Finish Week 6 brush tuning and diagnostics
Implemented the Week 6 multi-material brush work end-to-end: added marker chord-based stroke initialization, per-brush init overrides (`init_size_range`, `init_alpha_range`, `init_chord`), sampler/rasterizer wiring, and resume-time checks so ablation folders cannot mix different startup ranges. Updated brush defaults from tuning results, expanded tests around brush initialization/rasterizer/optimizer behavior, and extended comparison tooling with new scripts for marker diagnostics, cross-folder pairing, brush comparisons, and marker-chord plotting.

Also added the full Week 6 experiment outputs (ablation/tuning/held-out/fidelity/training runs), generated report figures and writeups for section 4.3, and updated `ROADMAP.md`/`CLAUDE.md` status and documentation to reflect completion.
</commit_message>
<xml_diff>
--- a/Bao_Cao_Tien_do.xlsx
+++ b/Bao_Cao_Tien_do.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\Painting_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054BA7D0-A795-4B5A-AF5C-F020F82CFA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C613AD-4492-4A46-8571-94C695376D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,18 +20,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>BÁO CÁO TIẾN ĐỘ THỰC HIỆN ĐỒ ÁN CƠ SỞ</t>
   </si>
   <si>
+    <t>Họ và tên sinh viên : Nguyễn Lê Hoàng - 24020003</t>
+  </si>
+  <si>
+    <t>Tên đề tài: Xây dựng hệ thống tái tạo tranh nghệ thuật từ ảnh thực tế bằng kỹ thuật cọ vẽ khả vi (Differentiable Neural Renderer)</t>
+  </si>
+  <si>
     <t>Tuần</t>
   </si>
   <si>
     <t>Ngày báo cáo</t>
   </si>
   <si>
-    <t>Nội dung theo kế họạch</t>
+    <t>04/09/2026</t>
+  </si>
+  <si>
+    <t>11/09/2026</t>
+  </si>
+  <si>
+    <t>18/09/2026</t>
+  </si>
+  <si>
+    <t>25/09/2026</t>
+  </si>
+  <si>
+    <t>02/10/2026</t>
+  </si>
+  <si>
+    <t>09/10/2026</t>
+  </si>
+  <si>
+    <t>Nội dung theo kế hoạch</t>
   </si>
   <si>
     <t>Nghiên cứu tổng quan và hoàn thiện đề cương:
@@ -53,6 +77,27 @@
 • Xây dựng chức năng cắt, chỉnh kích thước và chuẩn hóa ảnh đầu vào
 • Cài đặt bộ chia lưới (grid rendering) phục vụ xử lý ảnh kích thước lớn
 • Kiểm thử module tiền xử lý với tập ảnh mẫu</t>
+  </si>
+  <si>
+    <t>Cài đặt renderer khả vi và mô hình nét cọ cơ bản:
+• Cài đặt mạng Neural Renderer và nạp checkpoint sơn dầu có sẵn làm mốc so sánh
+• Xây dựng chương trình huấn luyện renderer trên dữ liệu nét cọ tổng hợp; huấn luyện renderer sơn dầu trên GPU RTX 3070
+• Sinh chuỗi tham số nét cọ ban đầu; thử render một nét cọ và kiểm tra lan truyền gradient (so sánh với sai phân hữu hạn)
+• Bổ sung ảnh tự chụp vào tập đánh giá; kiểm tra lại trên MacBook</t>
+  </si>
+  <si>
+    <t>Tối ưu hóa nét cọ theo ảnh gốc:
+• Cài đặt vòng lặp tối ưu hóa (optimization loop) sử dụng Pixel Loss và Sinkhorn Loss
+• Thử nghiệm ở chế độ toàn ảnh và chế độ chia nhỏ vùng (patch-based)
+• Đánh giá chất lượng tái tạo, tinh chỉnh trọng số các hàm mất mát
+• So sánh trực quan ảnh gốc và ảnh tái tạo ở giai đoạn này</t>
+  </si>
+  <si>
+    <t>Mở rộng đa chất liệu cọ vẽ:
+• Xây dựng bộ tham số riêng cho từng chất liệu: sơn dầu, màu nước, bút dạ, băng dính màu
+• Hiệu chỉnh đặc tính từng chất liệu (độ trong suốt, độ nhòe, hình dạng nét)
+• Kiểm thử và so sánh kết quả giữa các chất liệu trên cùng một ảnh
+• Cập nhật tài liệu kỹ thuật cho module render</t>
   </si>
   <si>
     <t>Nội dung thực tế đã thực hiện</t>
@@ -84,6 +129,35 @@
 • Viết mục Dữ liệu và tiền xử lý của chương Thực nghiệm, kèm hình minh họa quy trình tiền xử lý</t>
   </si>
   <si>
+    <t>• Cài đặt Neural Renderer cho 4 loại cọ: nhánh hình dạng (MLP + PixelShuffle) và nhánh màu (chuỗi ConvTranspose + BatchNorm), hợp nhất theo công thức ảnh nét = màu × mặt nạ, độ trong suốt = α × mặt nạ; có bản đầy đủ 128 px (18,1 triệu tham số) và bản nhẹ 32 px (5,4 triệu tham số)
+• Viết bộ chuyển đổi (adapter) nạp 8 checkpoint đã huấn luyện sẵn của tác giả gốc làm mốc so sánh: đầu ra trùng khớp hoàn toàn với mạng gốc (sai khác bằng 0 trên cả 8 checkpoint); nạp file ở chế độ an toàn, không thực thi mã tùy ý
+• Kiểm tra lan truyền gradient: so sánh đạo hàm tự động với sai phân hữu hạn (độ chính xác kép) cho mọi tham số nét cọ của 5 renderer (4 bản nhẹ và bản đầy đủ của cọ sơn dầu), sai số tương đối nhỏ hơn 10⁻⁵
+• Xây dựng chương trình huấn luyện renderer trên nét cọ ngẫu nhiên được vẽ tức thời bằng bộ vẽ thủ tục, theo đúng công thức của mã gốc (Adam 2×10⁻⁴, 50.000 nét/epoch, mất mát 100×MSE) để so sánh công bằng; sinh dữ liệu đa luồng (~1.800 nét/giây), chạy tiếp được từ checkpoint, ghi đường cong học và ảnh kiểm chứng
+• Huấn luyện renderer sơn dầu bản nhẹ trên GPU RTX 3070 (100 epoch, ~31 giây/epoch): trên 1.000 nét giữ lại (không dùng khi huấn luyện) đạt PSNR 24,16 dB, renderer gốc đạt 24,38 dB, chênh 0,22 dB (mục tiêu: không quá 1 dB)
+• Đo PSNR/SSIM của cả 8 renderer gốc trên cùng bộ 1.000 nét: lệch không quá 0,25 dB so với số liệu tác giả công bố, xác nhận quy trình đo; so sánh nét do mạng vẽ với bộ vẽ thủ tục bằng ảnh lưới kiểm chứng
+• Bổ sung 19 ảnh tự thu thập vào tập đánh giá (tổng 30 ảnh 512×512) và đóng băng lại (11 ảnh gốc giữ nguyên từng byte), thêm mô tả nội dung cho từng ảnh
+• Bổ sung 63 kiểm thử tự động (tổng 144, tất cả đạt); viết kịch bản kiểm tra thiết bị cho MacBook và kịch bản đo độ chính xác renderer; viết mục 4.1 (Neural renderer) của báo cáo</t>
+  </si>
+  <si>
+    <t>• Cài đặt hàm mất mát Sinkhorn (Optimal Transport), bộ lấy mẫu nét ban đầu (đặt ngẫu nhiên, ưu tiên vùng tranh còn khác ảnh gốc nhiều) và bộ tối ưu hóa nét cọ theo đúng vòng lặp của mã gốc: lấy mẫu nét, render, giãn/co 3×3 (làm kín mép nét, tránh viền tối), chồng lớp lên bức tranh, tính hàm mất mát, cập nhật tham số; giá trị và gradient Sinkhorn trùng với mã gốc
+• Hỗ trợ chế độ toàn ảnh và chia lưới cố định (chia nhỏ vùng); tính PSNR, SSIM và LPIPS (độ khác biệt theo cảm nhận thị giác, càng thấp càng tốt)
+• Viết công cụ chạy và thống kê thí nghiệm (so sánh theo cặp trên từng ảnh, khoảng tin cậy 95%, kiểm định Wilcoxon)
+• Thí nghiệm A: so sánh chỉ dùng Pixel Loss với Pixel + Sinkhorn (cọ sơn dầu, 500 nét, lưới 5×5, 30 ảnh × 2 cấu hình × 3 seed = 180 lần vẽ): PSNR 18,67 so với 18,69 dB, chênh lệch không có ý nghĩa thống kê; Sinkhorn làm thời gian tối ưu tăng 2,6 lần (từ 6,2 lên 16,0 giây mỗi bức tranh)
+• Thử trọng số Sinkhorn từ 0,1 đến 100 và tham số làm mịn ε từ 0,003 đến 0,1: không cải thiện; trọng số 100 hoặc ε lớn làm kết quả kém đi. Nguyên nhân: ở trọng số mặc định 0,1, gradient của Sinkhorn chỉ bằng 0,03–0,09% gradient của Pixel Loss
+• PSNR của chế độ lưới 5×5 cao hơn chế độ toàn ảnh 5,70 dB (cùng số nét, đúng trên cả 10 ảnh thử); bỏ phép giãn/co 3×3 làm PSNR giảm 2,71 dB; khởi tạo theo bản đồ sai số cho PSNR cao hơn 0,87 dB so với khởi tạo ngẫu nhiên phân bố đều
+• So với mã gốc 2021 (5 ảnh, cùng cách thu nhỏ ảnh đích): PSNR chỉ thấp hơn 0,02 dB (khoảng tin cậy 95%: −0,22 đến +0,17 dB), tức chất lượng tương đương mã gốc trong phạm vi sai số đo
+• Tính thêm LPIPS cho 699 bức tranh đã vẽ (không cần vẽ lại), kết quả cùng chiều với PSNR và SSIM; viết mục 4.2 của báo cáo (11 bảng số liệu, hình so sánh trực quan); bổ sung 77 kiểm thử tự động (tổng 221, tất cả đạt)</t>
+  </si>
+  <si>
+    <t>• Sửa lỗi cọ bút dạ không vẽ được: với cách khởi tạo của mã gốc (nét có độ dài bằng 0), renderer bản nhẹ không vẽ ra gì nên tranh gần như đen (4,2 dB); nay mỗi nét mới bắt đầu là một đoạn thẳng dài 0,4 cạnh ô lưới và tranh đạt khoảng 18–19 dB; vẫn giữ tùy chọn khởi tạo như mã gốc
+• Hiệu chỉnh đặc tính từng chất liệu theo quy trình thử trên 3 ảnh rồi kiểm tra lại trên 10 ảnh khác: nét ban đầu lớn hơn (kích thước 0,2–0,4 thay vì 0,1–0,25 như mã gốc) cho sơn dầu, màu nước, băng dính màu (+0,35 đến +0,39 dB); màu nước bắt đầu trong suốt hơn (hệ số α ban đầu 0,5–0,7 thay vì 0,98–1,0; +0,30 dB)
+• Huấn luyện renderer bản nhẹ cho màu nước, bút dạ, băng dính màu (100 epoch): PSNR trên 1.000 nét giữ lại kém renderer gốc lần lượt 0,45; 0,64 và 0,80 dB, đều đạt mục tiêu không quá 1 dB; băng dính màu huấn luyện đủ 400 epoch như mã gốc thì vượt renderer gốc 0,19 dB
+• So sánh 4 loại cọ trên cùng 3 ảnh (500 nét, 3 seed): PSNR băng dính màu 21,53 dB, sơn dầu 20,86, màu nước 20,36, bút dạ 19,41; băng dính màu cũng tốt nhất theo SSIM và LPIPS, còn ba loại kia được hai chỉ số này xếp khác với PSNR; lập hình so sánh dạng lưới 3 ảnh × 4 loại cọ; đo lại thời gian khi máy rảnh: tối ưu khoảng 5,8 giây mỗi tranh cho mọi loại cọ, cộng 0,9–1,4 giây vẽ ảnh cuối
+• Lặp lại thí nghiệm A (chỉ dùng Pixel Loss so với Pixel + Sinkhorn) cho 3 loại cọ còn lại (mỗi loại 10 ảnh × 2 cấu hình × 3 seed): PSNR chênh +0,04 (màu nước), −0,02 (bút dạ) và +0,05 dB (băng dính màu), không có ý nghĩa thống kê; Sinkhorn làm thời gian tối ưu tăng 2,6–2,7 lần
+• Vẽ bằng renderer tự huấn luyện: với màu nước và bút dạ, tranh tốt hơn khoảng 1,2 dB so với dùng renderer gốc (trung vị 0,7–0,8 dB)
+• Viết mục 4.3 (Chất liệu cọ vẽ) của báo cáo và tài liệu kỹ thuật module render; thêm công cụ so sánh và 14 kiểm thử tự động (tổng 235, tất cả đạt)</t>
+  </si>
+  <si>
     <t>Khó khăn, vướng mắc</t>
   </si>
   <si>
@@ -100,6 +174,28 @@
     <t>• Phải bảo đảm bộ vẽ nét cọ mới cho kết quả giống hệt mã gốc đến từng pixel; trong quá trình kiểm thử phát hiện thêm lỗi tương thích OpenCV 5 làm hỏng 3/4 loại cọ của mã gốc (đã sửa)
 • Tập ảnh đánh giá mới có 11 ảnh từ kho mã gốc; còn thiếu 10-20 ảnh tự chụp, cần bổ sung trước khi chạy thí nghiệm ở tuần 5
 • Chưa chạy lại bộ kiểm thử trên MacBook (MPS)</t>
+  </si>
+  <si>
+    <t>• Tuần 4 hoàn thành chậm so với kế hoạch (dự kiến 21–25/09, thực hiện đến 02/10)
+• Tốc độ huấn luyện bị giới hạn bởi bộ vẽ thủ tục chạy trên CPU (mỗi nét sơn dầu ~2,1 ms do phải xử lý ảnh kết cấu cọ 394×394), không phải bởi GPU; dùng nhiều tiến trình để nạp dữ liệu làm cạn bộ nhớ cam kết (commit) của Windows nên phải chuyển sang đa luồng trong một tiến trình
+• Phát hiện tham số độ trong suốt của cọ sơn dầu không làm đổi mặt nạ nhưng vẫn ảnh hưởng nhẹ (~1%) đến màu của nét, vì nhánh màu nhận toàn bộ tham số; sẽ cố định tham số này khi tối ưu
+• Kiểm tra trên MacBook (MPS) chỉ chạy được sau khi đẩy mã lên kho Git (02/10): 136 kiểm thử đạt, 8 kiểm thử bị bỏ qua vì máy chưa có checkpoint; trên MPS mới chạy thử huấn luyện 2 epoch nên chưa có đường cong học; renderer sơn dầu bản đầy đủ chưa huấn luyện lại (đang dùng checkpoint gốc, chỉ 43 epoch)</t>
+  </si>
+  <si>
+    <t>• Kết quả trái với giả thuyết ban đầu: Sinkhorn Loss gần như không cải thiện chất lượng mà làm chậm 2,3–2,6 lần; phải làm thêm 4 thí nghiệm ngoài kế hoạch (đo gradient, cách khởi tạo, phép giãn/co, so sánh với mã gốc) để giải thích
+• Phát hiện cọ bút dạ không thể bắt đầu vẽ với cách khởi tạo của mã gốc: ba điểm điều khiển của đường cong Bézier trùng nhau nên nét có độ dài bằng 0, không hiện gì và gradient bằng 0 (giải thích kết quả thấp bất thường 12–14 dB ở tuần 1); sẽ sửa ở tuần 6
+• Chạy lại cùng ảnh, cùng cấu hình, cùng seed trên GPU vẫn không cho kết quả giống hệt (thư viện cuDNN của NVIDIA có thể chọn thuật toán khác nhau giữa các lần chạy): PSNR chênh trung vị 0,10 dB, lớn nhất 0,85 dB, nên kết luận dựa trên giá trị trung bình; tốc độ máy bàn dao động tới 2 lần trong ngày nên chỉ so sánh thời gian đo cùng lúc
+• Chạy quá 2 tiến trình CUDA cùng lúc làm cạn bộ nhớ cam kết của Windows (một thí nghiệm bị dừng, phải chạy tiếp); Apple MPS không hỗ trợ phép gộp (pooling) khi kích thước vào không chia hết cho kích thước ra (32 → 24 px) nên phải viết lại phép thu nhỏ ảnh bằng phép nhân ma trận
+• Tuần 5 hoàn thành ngày 03/10 (LPIPS bổ sung ngày 05/10), sau ngày báo cáo 02/10; dự án đang chậm khoảng một tuần so với lịch ban đầu</t>
+  </si>
+  <si>
+    <t>• Huấn luyện renderer chậm vì bộ vẽ nét chạy trên CPU: 100 epoch mất 3,3 giờ với bút dạ và 2,2 giờ với màu nước (băng dính màu chỉ 14 phút)
+• Bộ nhớ cam kết (commit) của Windows bị cạn khi chạy 2 tiến trình PyTorch cùng lúc trong lúc đang mở nhiều chương trình khác (trình duyệt, Steam): hai tiến trình bị dừng, phải chạy tiếp từ điểm lưu, không mất kết quả; khi đóng bớt chương trình thì chạy được 3 tiến trình cùng lúc
+• Bước kiểm tra lại mã (review) phát hiện một lỗi trong cách đặt tâm nét bút dạ ban đầu; đã sửa và chạy lại toàn bộ thí nghiệm bút dạ, kết luận không đổi
+• Chưa giải thích được vì sao renderer tự huấn luyện của màu nước và bút dạ vẽ tốt hơn renderer gốc dù độ chính xác trên nét ngẫu nhiên thấp hơn
+• Không hiệu chỉnh độ nhòe (bộ vẽ nét gốc không có hiệu ứng này, thêm vào thì phải huấn luyện lại các renderer) và giữ số nét mặc định là 500; tuần này chỉ hiệu chỉnh cách nét bắt đầu (kích thước, độ trong suốt, độ dài nét bút dạ)
+• Lưới cố định để lộ các khe nền mảnh dọc biên giữa các ô (thấy rõ với bút dạ và băng dính màu trên nền đen); dự kiến chế độ chia lưới tăng dần ở tuần 7 sẽ che được, chưa kiểm chứng
+• Tuần 6 hoàn thành ngày 10/10, muộn một ngày so với ngày báo cáo 09/10; dự án đã theo kịp lịch ban đầu (tuần 7 theo lịch là 12–16/10)</t>
   </si>
   <si>
     <t>Kế hoạch tuần tiếp theo</t>
@@ -127,38 +223,6 @@
 • Bổ sung ảnh tự chụp vào tập đánh giá; kiểm tra lại trên MacBook</t>
   </si>
   <si>
-    <t>18/09/2026</t>
-  </si>
-  <si>
-    <t>Tên đề tài: Xây dựng hệ thống tái tạo tranh nghệ thuật từ ảnh thực tế bằng kỹ thuật cọ vẽ khả vi (Differentiable Neural Renderer)</t>
-  </si>
-  <si>
-    <t>Họ và tên sinh viên : Nguyễn Lê Hoàng - 24020003</t>
-  </si>
-  <si>
-    <t>Cài đặt renderer khả vi và mô hình nét cọ cơ bản:
-• Cài đặt mạng Neural Renderer và nạp checkpoint sơn dầu có sẵn làm mốc so sánh
-• Xây dựng chương trình huấn luyện renderer trên dữ liệu nét cọ tổng hợp; huấn luyện renderer sơn dầu trên GPU RTX 3070
-• Sinh chuỗi tham số nét cọ ban đầu; thử render một nét cọ và kiểm tra lan truyền gradient (so sánh với sai phân hữu hạn)
-• Bổ sung ảnh tự chụp vào tập đánh giá; kiểm tra lại trên MacBook</t>
-  </si>
-  <si>
-    <t>• Cài đặt Neural Renderer cho 4 loại cọ: nhánh hình dạng (MLP + PixelShuffle) và nhánh màu (chuỗi ConvTranspose + BatchNorm), hợp nhất theo công thức ảnh nét = màu × mặt nạ, độ trong suốt = α × mặt nạ; có bản đầy đủ 128 px (18,1 triệu tham số) và bản nhẹ 32 px (5,4 triệu tham số)
-• Viết bộ chuyển đổi (adapter) nạp 8 checkpoint đã huấn luyện sẵn của tác giả gốc làm mốc so sánh: đầu ra trùng khớp hoàn toàn với mạng gốc (sai khác bằng 0 trên cả 8 checkpoint); nạp file ở chế độ an toàn, không thực thi mã tùy ý
-• Kiểm tra lan truyền gradient: so sánh đạo hàm tự động với sai phân hữu hạn (độ chính xác kép) cho mọi tham số nét cọ của 5 renderer (4 bản nhẹ và bản đầy đủ của cọ sơn dầu), sai số tương đối nhỏ hơn 10⁻⁵
-• Xây dựng chương trình huấn luyện renderer trên nét cọ ngẫu nhiên được vẽ tức thời bằng bộ vẽ thủ tục, theo đúng công thức của mã gốc (Adam 2×10⁻⁴, 50.000 nét/epoch, mất mát 100×MSE) để so sánh công bằng; sinh dữ liệu đa luồng (~1.800 nét/giây), chạy tiếp được từ checkpoint, ghi đường cong học và ảnh kiểm chứng
-• Huấn luyện renderer sơn dầu bản nhẹ trên GPU RTX 3070 (100 epoch, ~31 giây/epoch): trên 1.000 nét giữ lại (không dùng khi huấn luyện) đạt PSNR [24,15] dB, renderer gốc đạt 24,38 dB, chênh [0,23] dB (mục tiêu: không quá 1 dB)
-• Đo PSNR/SSIM của cả 8 renderer gốc trên cùng bộ 1.000 nét: lệch không quá 0,25 dB so với số liệu tác giả công bố, xác nhận quy trình đo; so sánh nét do mạng vẽ với bộ vẽ thủ tục bằng ảnh lưới kiểm chứng
-• Bổ sung 19 ảnh tự thu thập vào tập đánh giá (tổng 30 ảnh 512×512) và đóng băng lại (11 ảnh gốc giữ nguyên từng byte), thêm mô tả nội dung cho từng ảnh
-• Bổ sung 63 kiểm thử tự động (tổng 144, tất cả đạt); viết kịch bản kiểm tra thiết bị cho MacBook và kịch bản đo độ chính xác renderer; viết mục 4.1 (Neural renderer) của báo cáo</t>
-  </si>
-  <si>
-    <t>• Tuần 4 hoàn thành chậm so với kế hoạch (dự kiến 21–25/09, thực hiện đến 02/10)
-• Tốc độ huấn luyện bị giới hạn bởi bộ vẽ thủ tục chạy trên CPU (mỗi nét sơn dầu ~2,1 ms do phải xử lý ảnh kết cấu cọ 394×394), không phải bởi GPU; dùng nhiều tiến trình để nạp dữ liệu làm cạn bộ nhớ cam kết (commit) của Windows nên phải chuyển sang đa luồng trong một tiến trình
-• Phát hiện tham số độ trong suốt của cọ sơn dầu không làm đổi mặt nạ nhưng vẫn ảnh hưởng nhẹ (~1%) đến màu của nét, vì nhánh màu nhận toàn bộ tham số; sẽ cố định tham số này khi tối ưu
-• Chưa chạy kiểm tra trên MacBook do mã mới chưa được đẩy lên kho Git; renderer sơn dầu bản đầy đủ chưa huấn luyện lại (đang dùng checkpoint gốc, chỉ 43 epoch)</t>
-  </si>
-  <si>
     <t>Tuần 5: Tối ưu hóa tham số nét cọ theo ảnh đích
 • Cài đặt Pixel Loss và Sinkhorn (Optimal Transport) Loss
 • Cài đặt bộ lấy mẫu nét theo bản đồ sai số và bộ tối ưu hóa tham số nét cọ cho từng khối ảnh
@@ -167,7 +231,23 @@
 • Chạy kiểm tra thiết bị trên MacBook và ghi lại kết quả</t>
   </si>
   <si>
-    <t>25/09/2026</t>
+    <t>Tuần 6: Mở rộng đa chất liệu cọ vẽ
+• Sửa cách khởi tạo nét bút dạ (độ dài nét ban đầu tối thiểu bằng 10% cạnh ô lưới, có tùy chọn giữ cách khởi tạo gốc)
+• Dùng lại hoặc huấn luyện renderer cho màu nước, bút dạ, băng dính màu; bổ sung các renderer tự huấn luyện vào bảng độ chính xác (renderer gốc của cả 4 loại cọ đã đo ở tuần 4)
+• Hiệu chỉnh đặc tính từng chất liệu (độ trong suốt, độ nhòe, hình dạng nét, số nét mặc định)
+• Vẽ cùng 3 ảnh với cả 4 loại cọ (500 nét), đo PSNR, SSIM, LPIPS và thời gian; lập hình so sánh dạng lưới 3 ảnh × 4 loại cọ
+• Viết mục Chất liệu cọ vẽ và cập nhật tài liệu kỹ thuật module render</t>
+  </si>
+  <si>
+    <t>Tuần 7: Hoàn thiện pipeline xử lý tự động
+• Cài đặt chế độ chia lưới tăng dần từ thô đến mịn (1×1 → 2×2 → … → M×M)
+• Viết lệnh chạy trọn quy trình từ ảnh đến tranh bằng một câu lệnh, có hiển thị tiến trình (số nét, hàm mất mát, thời gian)
+• So sánh chế độ chia lưới tăng dần với chế độ toàn ảnh và lưới cố định; đo chất lượng và thời gian theo số nét (100, 300, 500, 1000) cho từng loại cọ
+• Tối ưu tốc độ và bộ nhớ; đo hiệu năng trên các cấu hình phần cứng (CUDA, CPU, Apple MPS)
+• Kiểm thử pipeline end-to-end với nhiều ảnh; quyết định có dùng renderer tự huấn luyện làm mặc định cho màu nước và bút dạ hay không</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               </t>
   </si>
 </sst>
 </file>
@@ -259,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -268,10 +348,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -280,14 +369,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -623,72 +711,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:L10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="12" width="55" customWidth="1"/>
+    <col min="3" max="12" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="9" t="s">
+    <row r="1" spans="1:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
-    <row r="2" spans="2:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+    <row r="2" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
     </row>
-    <row r="3" spans="2:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="5"/>
+    <row r="3" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="4"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="11"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="1"/>
+      <c r="C5" s="6">
         <v>1</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="8"/>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1">
+      <c r="D5" s="6">
         <v>2</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="6">
         <v>3</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="6">
         <v>4</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="6">
         <v>5</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="6">
         <v>6</v>
       </c>
       <c r="I5" s="1">
@@ -704,116 +795,136 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="4">
-        <v>46121</v>
-      </c>
-      <c r="D6" s="4">
-        <v>46335</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>10</v>
+      </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="2:12" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="120" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
+        <v>14</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>17</v>
+      </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="2:12" ht="330" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="375" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
+      <c r="H8" s="8" t="s">
+        <v>24</v>
+      </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
     </row>
-    <row r="9" spans="2:12" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="270" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
+        <v>28</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
     </row>
-    <row r="10" spans="2:12" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="165" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>

</xml_diff>

<commit_message>
Week 7: progressive painter, pipeline defaults, benchmarks and report section 4.4
</commit_message>
<xml_diff>
--- a/Bao_Cao_Tien_do.xlsx
+++ b/Bao_Cao_Tien_do.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\Painting_project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\AppData\Local\Temp\claude\G--Github-Painting-project\6980c10e-80b9-456f-9e8f-50d072acc344\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C613AD-4492-4A46-8571-94C695376D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{837684E3-AE13-4538-9C53-1AB3A12AF62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+  <si>
+    <t xml:space="preserve">               </t>
+  </si>
   <si>
     <t>BÁO CÁO TIẾN ĐỘ THỰC HIỆN ĐỒ ÁN CƠ SỞ</t>
   </si>
@@ -53,6 +56,9 @@
   </si>
   <si>
     <t>09/10/2026</t>
+  </si>
+  <si>
+    <t>16/10/2026</t>
   </si>
   <si>
     <t>Nội dung theo kế hoạch</t>
@@ -98,6 +104,13 @@
 • Hiệu chỉnh đặc tính từng chất liệu (độ trong suốt, độ nhòe, hình dạng nét)
 • Kiểm thử và so sánh kết quả giữa các chất liệu trên cùng một ảnh
 • Cập nhật tài liệu kỹ thuật cho module render</t>
+  </si>
+  <si>
+    <t>Hoàn thiện pipeline xử lý tự động:
+• Kết nối toàn bộ pipeline: nhận ảnh → tiền xử lý → chia lưới → tối ưu nét cọ → kết xuất tranh
+• Cài đặt thanh tiến trình hiển thị quá trình xử lý theo thời gian thực
+• Tối ưu hiệu năng xử lý (tốc độ, bộ nhớ) trên các cấu hình phần cứng khác nhau
+• Kiểm thử pipeline end-to-end với nhiều ảnh đầu vào</t>
   </si>
   <si>
     <t>Nội dung thực tế đã thực hiện</t>
@@ -158,6 +171,16 @@
 • Viết mục 4.3 (Chất liệu cọ vẽ) của báo cáo và tài liệu kỹ thuật module render; thêm công cụ so sánh và 14 kiểm thử tự động (tổng 235, tất cả đạt)</t>
   </si>
   <si>
+    <t>• Rà soát lại mã trước khi viết mã mới: sửa 4 lỗi nhỏ trong các script thí nghiệm; sau đó phát hiện và sửa thêm lỗi ảnh xám 16-bit bị đọc thành gần như trắng
+• Cài đặt chế độ chia lưới tăng dần từ thô đến mịn (1×1 → 5×5), dùng chung một đường xử lý với lưới cố định và toàn ảnh; kết quả khớp với mã gốc demo_prog.py (chênh −0,05 dB, không đáng kể)
+• Lệnh run_paint.py chạy trọn quy trình từ ảnh đến tranh bằng một câu lệnh, có dòng tiến trình cập nhật theo thời gian thực (cấp lưới, số nét, hàm mất mát, PSNR, thời gian); báo lỗi rõ ràng khi ảnh hỏng, sai định dạng hoặc quá lớn
+• So sánh 3 chế độ chia lưới (10 ảnh × 3 seed): lưới tăng dần tốt hơn lưới cố định +0,25 dB với sơn dầu và +1,1 đến +2,1 dB với màu nước, bút dạ, băng dính màu (che được các khe nền dọc biên ô lưới); chế độ toàn ảnh kém hơn 6,5 dB
+• Lịch tốc độ học dạng cosine: tốt hơn +0,07 đến +0,32 dB nên được dùng làm mặc định; phân bổ nét theo sai số và tính toán bfloat16 giữ làm tùy chọn
+• Khảo sát số nét 100/300/500/1000 cho 4 loại cọ: chất lượng gần bão hòa ở khoảng 500 nét (trừ băng dính màu); thời gian 9–17 giây trên GPU
+• Đo hiệu năng: GPU 12 giây/tranh, CPU 130 giây/tranh, bộ nhớ dưới 0,4 GB; kiểm thử end-to-end với 20 ảnh đầu vào (nhiều kích thước, tỉ lệ, định dạng): tất cả đạt
+• Viết mục 4.4 của báo cáo kèm sơ đồ pipeline; 253 kiểm thử tự động đều đạt</t>
+  </si>
+  <si>
     <t>Khó khăn, vướng mắc</t>
   </si>
   <si>
@@ -198,6 +221,12 @@
 • Tuần 6 hoàn thành ngày 10/10, muộn một ngày so với ngày báo cáo 09/10; dự án đã theo kịp lịch ban đầu (tuần 7 theo lịch là 12–16/10)</t>
   </si>
   <si>
+    <t>• Windows 11 tự giảm tốc các tiến trình chạy nền (power throttling): CPU chậm 3,5–3,9 lần, GPU chậm tới 1,8 lần; đã tắt cơ chế này trong mọi script; số đo thời gian của tuần 5–6 vì vậy chỉ nên so sánh tương đối
+• torch.compile không dùng được trên Windows (thiếu Triton); bfloat16 nhanh hơn 25% ở lưới cố định nhưng chậm hơn ở chế độ tăng dần và làm màu nước kém 0,13 dB, nên không dùng mặc định
+• Renderer bản đầy đủ cần tới 6,8 GB bộ nhớ GPU với 1000 nét ở lưới cố định (gần giới hạn 8 GB); thời gian chạy của nó dao động mạnh giữa các lần
+• Chưa đo trên MacBook (mps và CPU của M4): cần chạy benchmark.py trên MacBook</t>
+  </si>
+  <si>
     <t>Kế hoạch tuần tiếp theo</t>
   </si>
   <si>
@@ -247,7 +276,11 @@
 • Kiểm thử pipeline end-to-end với nhiều ảnh; quyết định có dùng renderer tự huấn luyện làm mặc định cho màu nước và bút dạ hay không</t>
   </si>
   <si>
-    <t xml:space="preserve">               </t>
+    <t>Tuần 8: Xây dựng giao diện người dùng
+• Thiết kế và cài đặt giao diện Web App (Gradio): tải ảnh, chọn chất liệu cọ, số nét, chế độ chia lưới
+• Hiển thị thanh tiến trình và tranh đang vẽ theo thời gian thực; so sánh ảnh gốc và tranh hoàn thiện
+• Tệp khởi động bằng nhấp đúp, không cần gõ lệnh
+• Kiểm thử tương tác người dùng, sửa lỗi giao diện; chạy benchmark trên MacBook</t>
   </si>
 </sst>
 </file>
@@ -721,10 +754,10 @@
   <sheetData>
     <row r="1" spans="1:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -732,7 +765,7 @@
     </row>
     <row r="2" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="16" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -740,7 +773,7 @@
     </row>
     <row r="3" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="14" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
@@ -750,7 +783,7 @@
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
       <c r="C4" s="9" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -797,135 +830,145 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I6" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>12</v>
+      </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" ht="120" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" s="1"/>
+        <v>19</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>20</v>
+      </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" ht="375" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I8" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>28</v>
+      </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
     </row>
     <row r="9" spans="1:12" ht="270" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="I9" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>36</v>
+      </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
     </row>
     <row r="10" spans="1:12" ht="165" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>44</v>
+      </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -938,6 +981,6 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>